<commit_message>
更新 modify.xlsx 和 remove.xlsx 数据文件
</commit_message>
<xml_diff>
--- a/data/remove.xlsx
+++ b/data/remove.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>20261009000001</t>
+          <t>20261014000001</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -600,7 +600,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20261009000002</t>
+          <t>20261014000002</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -648,7 +648,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>20261009000003</t>
+          <t>20261014000003</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -696,7 +696,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>20261009000004</t>
+          <t>20261014000004</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -744,7 +744,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>20261009000005</t>
+          <t>20261014000005</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -792,7 +792,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>20261009000006</t>
+          <t>20261014000006</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -840,7 +840,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>20261009000007</t>
+          <t>20261014000007</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20261009000008</t>
+          <t>20261014000008</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -936,7 +936,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>20261009000009</t>
+          <t>20261014000009</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>20261009000010</t>
+          <t>20261014000010</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>20261009000011</t>
+          <t>20261014000011</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>20261009000012</t>
+          <t>20261014000012</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>20261009000013</t>
+          <t>20261014000013</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>20261009000014</t>
+          <t>20261014000014</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>20261009000015</t>
+          <t>20261014000015</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>20261009000016</t>
+          <t>20261014000016</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>20261009000017</t>
+          <t>20261014000017</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>20261009000018</t>
+          <t>20261014000018</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>20261009000019</t>
+          <t>20261014000019</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>20261009000020</t>
+          <t>20261014000020</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>20261009000021</t>
+          <t>20261014000021</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>20261009000022</t>
+          <t>20261014000022</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>20261009000023</t>
+          <t>20261014000023</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>20261009000024</t>
+          <t>20261014000024</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>20261009000025</t>
+          <t>20261014000025</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>20261009000026</t>
+          <t>20261014000026</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>20261009000027</t>
+          <t>20261014000027</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>20261009000028</t>
+          <t>20261014000028</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>20261009000029</t>
+          <t>20261014000029</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>20261009000030</t>
+          <t>20261014000030</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>20261009000031</t>
+          <t>20261014000031</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>20261009000032</t>
+          <t>20261014000032</t>
         </is>
       </c>
       <c r="J33" t="inlineStr"/>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>20261009000033</t>
+          <t>20261014000033</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>20261009000034</t>
+          <t>20261014000034</t>
         </is>
       </c>
       <c r="J35" t="inlineStr"/>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>20261009000035</t>
+          <t>20261014000035</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>20261009000036</t>
+          <t>20261014000036</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>20261009000037</t>
+          <t>20261014000037</t>
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>20261009000038</t>
+          <t>20261014000038</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>20261009000039</t>
+          <t>20261014000039</t>
         </is>
       </c>
       <c r="J40" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>20261009000040</t>
+          <t>20261014000040</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>20261009000041</t>
+          <t>20261014000041</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>20261009000042</t>
+          <t>20261014000042</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>20261009000043</t>
+          <t>20261014000043</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>20261009000044</t>
+          <t>20261014000044</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>20261009000045</t>
+          <t>20261014000045</t>
         </is>
       </c>
       <c r="J46" t="inlineStr"/>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>20261009000046</t>
+          <t>20261014000046</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>20261009000047</t>
+          <t>20261014000047</t>
         </is>
       </c>
       <c r="J48" t="inlineStr"/>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>20261009000048</t>
+          <t>20261014000048</t>
         </is>
       </c>
       <c r="J49" t="inlineStr"/>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>20261009000049</t>
+          <t>20261014000049</t>
         </is>
       </c>
       <c r="J50" t="inlineStr"/>
@@ -2904,7 +2904,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>20261009000050</t>
+          <t>20261014000050</t>
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>20261009000051</t>
+          <t>20261014000051</t>
         </is>
       </c>
       <c r="J52" t="inlineStr"/>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>20261009000052</t>
+          <t>20261014000052</t>
         </is>
       </c>
       <c r="J53" t="inlineStr"/>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>20261009000053</t>
+          <t>20261014000053</t>
         </is>
       </c>
       <c r="J54" t="inlineStr"/>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>20261009000054</t>
+          <t>20261014000054</t>
         </is>
       </c>
       <c r="J55" t="inlineStr"/>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>20261009000055</t>
+          <t>20261014000055</t>
         </is>
       </c>
       <c r="J56" t="inlineStr"/>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>20261009000056</t>
+          <t>20261014000056</t>
         </is>
       </c>
       <c r="J57" t="inlineStr"/>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>20261009000057</t>
+          <t>20261014000057</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>20261009000058</t>
+          <t>20261014000058</t>
         </is>
       </c>
       <c r="J59" t="inlineStr"/>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>20261009000059</t>
+          <t>20261014000059</t>
         </is>
       </c>
       <c r="J60" t="inlineStr"/>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>20261009000060</t>
+          <t>20261014000060</t>
         </is>
       </c>
       <c r="J61" t="inlineStr"/>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>20261009000061</t>
+          <t>20261014000061</t>
         </is>
       </c>
       <c r="J62" t="inlineStr"/>
@@ -3480,7 +3480,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>20261009000062</t>
+          <t>20261014000062</t>
         </is>
       </c>
       <c r="J63" t="inlineStr"/>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>20261009000063</t>
+          <t>20261014000063</t>
         </is>
       </c>
       <c r="J64" t="inlineStr"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>20261009000064</t>
+          <t>20261014000064</t>
         </is>
       </c>
       <c r="J65" t="inlineStr"/>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>20261009000065</t>
+          <t>20261014000065</t>
         </is>
       </c>
       <c r="J66" t="inlineStr"/>
@@ -3672,7 +3672,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>20261009000066</t>
+          <t>20261014000066</t>
         </is>
       </c>
       <c r="J67" t="inlineStr"/>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>20261009000067</t>
+          <t>20261014000067</t>
         </is>
       </c>
       <c r="J68" t="inlineStr"/>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>20261009000068</t>
+          <t>20261014000068</t>
         </is>
       </c>
       <c r="J69" t="inlineStr"/>
@@ -3816,7 +3816,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>20261009000069</t>
+          <t>20261014000069</t>
         </is>
       </c>
       <c r="J70" t="inlineStr"/>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>20261009000070</t>
+          <t>20261014000070</t>
         </is>
       </c>
       <c r="J71" t="inlineStr"/>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>20261009000071</t>
+          <t>20261014000071</t>
         </is>
       </c>
       <c r="J72" t="inlineStr"/>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>20261009000072</t>
+          <t>20261014000072</t>
         </is>
       </c>
       <c r="J73" t="inlineStr"/>
@@ -4008,7 +4008,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>20261009000073</t>
+          <t>20261014000073</t>
         </is>
       </c>
       <c r="J74" t="inlineStr"/>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>20261009000074</t>
+          <t>20261014000074</t>
         </is>
       </c>
       <c r="J75" t="inlineStr"/>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>20261009000075</t>
+          <t>20261014000075</t>
         </is>
       </c>
       <c r="J76" t="inlineStr"/>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>20261009000076</t>
+          <t>20261014000076</t>
         </is>
       </c>
       <c r="J77" t="inlineStr"/>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>20261009000077</t>
+          <t>20261014000077</t>
         </is>
       </c>
       <c r="J78" t="inlineStr"/>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>20261009000078</t>
+          <t>20261014000078</t>
         </is>
       </c>
       <c r="J79" t="inlineStr"/>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>20261009000079</t>
+          <t>20261014000079</t>
         </is>
       </c>
       <c r="J80" t="inlineStr"/>
@@ -4344,7 +4344,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>20261009000080</t>
+          <t>20261014000080</t>
         </is>
       </c>
       <c r="J81" t="inlineStr"/>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>20261009000081</t>
+          <t>20261014000081</t>
         </is>
       </c>
       <c r="J82" t="inlineStr"/>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>20261009000082</t>
+          <t>20261014000082</t>
         </is>
       </c>
       <c r="J83" t="inlineStr"/>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>20261009000083</t>
+          <t>20261014000083</t>
         </is>
       </c>
       <c r="J84" t="inlineStr"/>
@@ -4536,7 +4536,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>20261009000084</t>
+          <t>20261014000084</t>
         </is>
       </c>
       <c r="J85" t="inlineStr"/>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>20261009000085</t>
+          <t>20261014000085</t>
         </is>
       </c>
       <c r="J86" t="inlineStr"/>
@@ -4632,7 +4632,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>20261009000086</t>
+          <t>20261014000086</t>
         </is>
       </c>
       <c r="J87" t="inlineStr"/>
@@ -4680,7 +4680,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>20261009000087</t>
+          <t>20261014000087</t>
         </is>
       </c>
       <c r="J88" t="inlineStr"/>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>20261009000088</t>
+          <t>20261014000088</t>
         </is>
       </c>
       <c r="J89" t="inlineStr"/>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>20261009000089</t>
+          <t>20261014000089</t>
         </is>
       </c>
       <c r="J90" t="inlineStr"/>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>20261009000090</t>
+          <t>20261014000090</t>
         </is>
       </c>
       <c r="J91" t="inlineStr"/>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>20261009000091</t>
+          <t>20261014000091</t>
         </is>
       </c>
       <c r="J92" t="inlineStr"/>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>20261009000092</t>
+          <t>20261014000092</t>
         </is>
       </c>
       <c r="J93" t="inlineStr"/>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>20261009000093</t>
+          <t>20261014000093</t>
         </is>
       </c>
       <c r="J94" t="inlineStr"/>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>20261009000094</t>
+          <t>20261014000094</t>
         </is>
       </c>
       <c r="J95" t="inlineStr"/>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>20261009000095</t>
+          <t>20261014000095</t>
         </is>
       </c>
       <c r="J96" t="inlineStr"/>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>20261009000096</t>
+          <t>20261014000096</t>
         </is>
       </c>
       <c r="J97" t="inlineStr"/>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>20261009000097</t>
+          <t>20261014000097</t>
         </is>
       </c>
       <c r="J98" t="inlineStr"/>
@@ -5208,7 +5208,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>20261009000098</t>
+          <t>20261014000098</t>
         </is>
       </c>
       <c r="J99" t="inlineStr"/>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>20261009000099</t>
+          <t>20261014000099</t>
         </is>
       </c>
       <c r="J100" t="inlineStr"/>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>20261009000100</t>
+          <t>20261014000100</t>
         </is>
       </c>
       <c r="J101" t="inlineStr"/>

</xml_diff>